<commit_message>
FET: added original Sormani data
</commit_message>
<xml_diff>
--- a/RRMS.xlsx
+++ b/RRMS.xlsx
@@ -8,22 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebmhealth-my.sharepoint.com/personal/ananda_biswas_ebmhealth_in/Documents/Documents/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D706924-52C5-49A0-BC0F-B6C314943939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{6D706924-52C5-49A0-BC0F-B6C314943939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60F50B93-ADFE-418E-BDAD-B14665402FC7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="RRMS Data" sheetId="1" r:id="rId1"/>
     <sheet name="Description" sheetId="4" r:id="rId2"/>
     <sheet name="Abbreviations" sheetId="2" r:id="rId3"/>
     <sheet name="References" sheetId="3" r:id="rId4"/>
+    <sheet name="Sormani Data" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="121">
   <si>
     <t>Study</t>
   </si>
@@ -52,9 +66,6 @@
     <t>DPRR</t>
   </si>
   <si>
-    <t>DPRR.lower</t>
-  </si>
-  <si>
     <t>DPRR.upper</t>
   </si>
   <si>
@@ -133,21 +144,9 @@
     <t>O'Connor (2)</t>
   </si>
   <si>
-    <t>IFNbeta-1b 1.6 MIU vs PBO</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 8 MIU vs PBO</t>
-  </si>
-  <si>
-    <t>MMPS vs PBO</t>
-  </si>
-  <si>
     <t>GA vs PBO</t>
   </si>
   <si>
-    <t>IFNbeta-1a 6 MIU vs PBO</t>
-  </si>
-  <si>
     <t>IVIg vs PBO</t>
   </si>
   <si>
@@ -157,48 +156,15 @@
     <t>Hydrolytic enzymes vs PBO</t>
   </si>
   <si>
-    <t>NAT vs PBO</t>
-  </si>
-  <si>
     <t>Cladribine 3.5 mg/kg vs PBO</t>
   </si>
   <si>
     <t>Cladribine 5.25 mg/kg vs PBO</t>
   </si>
   <si>
-    <t>IFNbeta-1a and oral MPS vs IFNbeta-1a and PBO</t>
-  </si>
-  <si>
-    <t>IFNbeta1b vs IFNbeta1a</t>
-  </si>
-  <si>
-    <t>NAT + IFNbeta-1a vs IFNbeta-1a</t>
-  </si>
-  <si>
-    <t>ALE 12 mg vs IFNbeta-1a</t>
-  </si>
-  <si>
-    <t>ALE 24 mg vs IFNbeta-1a</t>
-  </si>
-  <si>
-    <t>IFNbeta vs GA</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 1.6 MIU</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 8 MIU</t>
-  </si>
-  <si>
-    <t>MMPS</t>
-  </si>
-  <si>
     <t>GA</t>
   </si>
   <si>
-    <t>IFNbeta-1a 6 MIU</t>
-  </si>
-  <si>
     <t>IVIg</t>
   </si>
   <si>
@@ -208,97 +174,19 @@
     <t>Hydrolytic enzymes</t>
   </si>
   <si>
-    <t>NAT</t>
-  </si>
-  <si>
     <t>Cladribine 3.5 mg/kg</t>
   </si>
   <si>
     <t>Cladribine 5.25 mg/kg</t>
   </si>
   <si>
-    <t>IFNbeta-1a and oral MPS</t>
-  </si>
-  <si>
-    <t>IFNbeta1b</t>
-  </si>
-  <si>
-    <t>NAT + IFNbeta-1a</t>
-  </si>
-  <si>
-    <t>ALE 12 mg</t>
-  </si>
-  <si>
-    <t>ALE 24 mg</t>
-  </si>
-  <si>
-    <t>IFNbeta</t>
-  </si>
-  <si>
     <t>PBO</t>
   </si>
   <si>
-    <t>IFNbeta-1a and PBO</t>
-  </si>
-  <si>
-    <t>IFNbeta1a</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a</t>
-  </si>
-  <si>
     <t>Study.Year</t>
   </si>
   <si>
     <t>Treatment.Contrast</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 60 mcg</t>
-  </si>
-  <si>
-    <t>30mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 60 mcg vs 30mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 30 mcg + AZA 50 mg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 30 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 30 mcg + AZA 50 mg vs IFNbeta-1a 30 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 30 mcg IM + AZA 50 mg + prednisone 10 mg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1a 30 mcg IM + AZA 50 mg + prednisone 10 mg vs IFNbeta-1a 30 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 250 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 250 mcg vs GA</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 500 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta-1b 500 mcg vs GA</t>
-  </si>
-  <si>
-    <t>IFNbeta 22 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta 22 mcg vs PBO</t>
-  </si>
-  <si>
-    <t>IFNbeta 44 mcg</t>
-  </si>
-  <si>
-    <t>IFNbeta 44 mcg vs PBO</t>
   </si>
   <si>
     <t>mcg</t>
@@ -431,12 +319,162 @@
   <si>
     <t xml:space="preserve">Sormani, Maria Pia &amp; Bonzano, L &amp; Roccatagliata, L &amp; Mancardi, G &amp; Uccelli, Antonio &amp; Bruzzi, Paolo. (2010). Surrogate endpoints for EDSS worsening in multiple sclerosis A meta-analytic approach. Neurology. 75. 302-9. 10.1212/WNL.0b013e3181ea15aa. </t>
   </si>
+  <si>
+    <t>IFNβ-1b 1.6 MIU vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 8 MIU vs PBO</t>
+  </si>
+  <si>
+    <t>Methylprednisolone vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 6 MIU vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 22 μg vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 44 μg vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 44 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 22 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 6 MIU</t>
+  </si>
+  <si>
+    <t>Methylprednisolone</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 8 MIU</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 1.6 MIU</t>
+  </si>
+  <si>
+    <t>Natalizumab vs PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a and oral methylprednisolone vs IFNβ-1a and PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 60 μg vs 30 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1b vs IFNβ-1a</t>
+  </si>
+  <si>
+    <t>Natalizumab + IFNβ-1a vs IFNβ-1a</t>
+  </si>
+  <si>
+    <t>Alemtuzumab 12 mg vs IFNβ-1a</t>
+  </si>
+  <si>
+    <t>Alemtuzumab 24 mg vs IFNβ-1a</t>
+  </si>
+  <si>
+    <t>IFNβ vs GA</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 30 μg plus AZA 50 mg vs IFNβ-1a 30 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 30 μg IM plus AZA 50 mg plus prednisone 10 mg vs IFNβ-1a 30 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 250 μg vs GA</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 500 μg vs GA</t>
+  </si>
+  <si>
+    <t>Natalizumab</t>
+  </si>
+  <si>
+    <t>IFNβ-1a and oral methylprednisolone</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 60 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1b</t>
+  </si>
+  <si>
+    <t>Natalizumab + IFNβ-1a</t>
+  </si>
+  <si>
+    <t>Alemtuzumab 12 mg</t>
+  </si>
+  <si>
+    <t>Alemtuzumab 24 mg</t>
+  </si>
+  <si>
+    <t>IFNβ</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 30 μg plus AZA 50 mg</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 30 μg IM plus AZA 50 mg plus prednisone 10 mg</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 250 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1b 500 μg</t>
+  </si>
+  <si>
+    <t>IFNβ-1a and PBO</t>
+  </si>
+  <si>
+    <t>IFNβ-1a</t>
+  </si>
+  <si>
+    <t>IFNβ-1a 30 μg</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>ARR control arm</t>
+  </si>
+  <si>
+    <t>ARR experimental arm</t>
+  </si>
+  <si>
+    <t>REL-effect</t>
+  </si>
+  <si>
+    <t>Disability control arm</t>
+  </si>
+  <si>
+    <t>Disability experimental arm</t>
+  </si>
+  <si>
+    <t>DIS-effect</t>
+  </si>
+  <si>
+    <t>DPRR.lower</t>
+  </si>
+  <si>
+    <t>Treatment effect on disability</t>
+  </si>
+  <si>
+    <t>Treatment effect on annualised relapse rate</t>
+  </si>
+  <si>
+    <t>RRMS Data is the one reported in NICE DSU TSD 20. Sormani Data is the one reported in the original paper by Sormani et. al.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -476,6 +514,14 @@
       <sz val="11"/>
       <color rgb="FF00B050"/>
       <name val="Congenial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -519,7 +565,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -536,6 +582,16 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -847,13 +903,13 @@
   <cols>
     <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="72.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="63" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -862,16 +918,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>75</v>
+      <c r="E1" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -892,27 +948,27 @@
         <v>8</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>1993</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="F2">
         <v>248</v>
@@ -941,19 +997,19 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>1993</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="F3">
         <v>247</v>
@@ -982,19 +1038,19 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>1994</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="F4">
         <v>26</v>
@@ -1023,19 +1079,19 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>1995</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F5">
         <v>251</v>
@@ -1064,19 +1120,19 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>1996</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="F6">
         <v>172</v>
@@ -1105,19 +1161,19 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>1997</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F7">
         <v>150</v>
@@ -1146,19 +1202,19 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>1997</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F8">
         <v>51</v>
@@ -1187,19 +1243,19 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>1998</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F9">
         <v>40</v>
@@ -1228,19 +1284,19 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>1998</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="F10">
         <v>376</v>
@@ -1269,19 +1325,19 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>1998</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="F11">
         <v>371</v>
@@ -1310,19 +1366,19 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>2005</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F12">
         <v>306</v>
@@ -1351,19 +1407,19 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>2006</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="F13">
         <v>942</v>
@@ -1392,19 +1448,19 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>2009</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F14">
         <v>870</v>
@@ -1433,19 +1489,19 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15">
         <v>2009</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F15">
         <v>893</v>
@@ -1474,19 +1530,19 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>2009</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="D16" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="F16">
         <v>130</v>
@@ -1515,19 +1571,19 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>2002</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="D17" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="E17" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F17">
         <v>802</v>
@@ -1556,19 +1612,19 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>2002</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="E18" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
       <c r="F18">
         <v>188</v>
@@ -1597,19 +1653,19 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19">
         <v>2006</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="F19">
         <v>1171</v>
@@ -1638,19 +1694,19 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>2008</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="E20" t="s">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="F20">
         <v>223</v>
@@ -1679,19 +1735,19 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21">
         <v>2008</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>101</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="E21" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="F21">
         <v>221</v>
@@ -1720,19 +1776,19 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22">
         <v>2008</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="D22" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="F22">
         <v>764</v>
@@ -1761,19 +1817,19 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23">
         <v>2009</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E23" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="F23">
         <v>118</v>
@@ -1802,19 +1858,19 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24">
         <v>2009</v>
       </c>
       <c r="C24" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E24" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F24">
         <v>123</v>
@@ -1843,19 +1899,19 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25">
         <v>2009</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="D25" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F25">
         <v>1345</v>
@@ -1884,19 +1940,19 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26">
         <v>2009</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="D26" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="E26" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F26">
         <v>1347</v>
@@ -1930,7 +1986,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C45CA802-2779-4F18-8B64-B2B0BF5BE6B5}">
-  <dimension ref="A2"/>
+  <dimension ref="A2:A4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="103.1796875" customWidth="1"/>
@@ -1938,7 +1994,12 @@
   <sheetData>
     <row r="2" spans="1:1" ht="206" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>109</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1948,32 +2009,32 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ABC7DA4-7B42-4D10-ADBF-E0BA6280D7A9}">
-  <dimension ref="A5:B17"/>
+  <dimension ref="A5:B19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:2" ht="24.5" x14ac:dyDescent="0.65">
       <c r="A5" s="2" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1981,7 +2042,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1989,63 +2050,79 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>105</v>
+      <c r="B19" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2064,17 +2141,1174 @@
   <sheetData>
     <row r="5" spans="1:2" ht="24.5" x14ac:dyDescent="0.65">
       <c r="A5" s="2" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="B8" s="5" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B11" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{630BD9AE-3F46-4DCB-B3A5-7C82CA80C9C1}">
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="63" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="8"/>
+    <col min="9" max="9" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>112</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>1993</v>
+      </c>
+      <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2">
+        <v>248</v>
+      </c>
+      <c r="G2">
+        <v>24</v>
+      </c>
+      <c r="H2" s="8">
+        <v>323</v>
+      </c>
+      <c r="I2">
+        <v>1.27</v>
+      </c>
+      <c r="J2">
+        <v>1.17</v>
+      </c>
+      <c r="K2">
+        <v>0.92</v>
+      </c>
+      <c r="L2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="M2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>1993</v>
+      </c>
+      <c r="C3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3">
+        <v>247</v>
+      </c>
+      <c r="G3">
+        <v>24</v>
+      </c>
+      <c r="H3" s="8">
+        <v>321</v>
+      </c>
+      <c r="I3">
+        <v>1.27</v>
+      </c>
+      <c r="J3">
+        <v>0.84</v>
+      </c>
+      <c r="K3">
+        <v>0.66</v>
+      </c>
+      <c r="L3">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="M3">
+        <v>0.2</v>
+      </c>
+      <c r="N3">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>1994</v>
+      </c>
+      <c r="C4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4">
+        <v>26</v>
+      </c>
+      <c r="G4">
+        <v>24</v>
+      </c>
+      <c r="H4" s="8">
+        <v>37</v>
+      </c>
+      <c r="I4">
+        <v>0.72</v>
+      </c>
+      <c r="J4">
+        <v>0.59</v>
+      </c>
+      <c r="K4">
+        <v>0.81</v>
+      </c>
+      <c r="L4">
+        <v>0.22</v>
+      </c>
+      <c r="M4">
+        <v>0.25</v>
+      </c>
+      <c r="N4">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>1995</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5">
+        <v>251</v>
+      </c>
+      <c r="G5">
+        <v>24</v>
+      </c>
+      <c r="H5" s="8">
+        <v>355</v>
+      </c>
+      <c r="I5">
+        <v>0.84</v>
+      </c>
+      <c r="J5">
+        <v>0.6</v>
+      </c>
+      <c r="K5">
+        <v>0.71</v>
+      </c>
+      <c r="L5">
+        <v>0.25</v>
+      </c>
+      <c r="M5">
+        <v>0.22</v>
+      </c>
+      <c r="N5">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1996</v>
+      </c>
+      <c r="C6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6">
+        <v>172</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6" s="8">
+        <v>243</v>
+      </c>
+      <c r="I6">
+        <v>0.9</v>
+      </c>
+      <c r="J6">
+        <v>0.61</v>
+      </c>
+      <c r="K6">
+        <v>0.68</v>
+      </c>
+      <c r="L6">
+        <v>0.33</v>
+      </c>
+      <c r="M6">
+        <v>0.21</v>
+      </c>
+      <c r="N6">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>1997</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7">
+        <v>150</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7" s="8">
+        <v>212</v>
+      </c>
+      <c r="I7">
+        <v>1.26</v>
+      </c>
+      <c r="J7">
+        <v>0.52</v>
+      </c>
+      <c r="K7">
+        <v>0.41</v>
+      </c>
+      <c r="L7">
+        <v>0.23</v>
+      </c>
+      <c r="M7">
+        <v>0.16</v>
+      </c>
+      <c r="N7">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>1997</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8">
+        <v>51</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8" s="8">
+        <v>72</v>
+      </c>
+      <c r="I8">
+        <v>1.31</v>
+      </c>
+      <c r="J8">
+        <v>0.45</v>
+      </c>
+      <c r="K8">
+        <v>0.34</v>
+      </c>
+      <c r="L8">
+        <v>0.37</v>
+      </c>
+      <c r="M8">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="N8">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>1998</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9">
+        <v>40</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9" s="8">
+        <v>57</v>
+      </c>
+      <c r="I9">
+        <v>1.61</v>
+      </c>
+      <c r="J9">
+        <v>0.59</v>
+      </c>
+      <c r="K9">
+        <v>0.37</v>
+      </c>
+      <c r="L9">
+        <v>0.17</v>
+      </c>
+      <c r="M9">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="N9">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>1998</v>
+      </c>
+      <c r="C10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10">
+        <v>376</v>
+      </c>
+      <c r="G10">
+        <v>24</v>
+      </c>
+      <c r="H10" s="8">
+        <v>400</v>
+      </c>
+      <c r="I10">
+        <v>1.28</v>
+      </c>
+      <c r="J10">
+        <v>0.91</v>
+      </c>
+      <c r="K10">
+        <v>0.71</v>
+      </c>
+      <c r="L10">
+        <v>0.37</v>
+      </c>
+      <c r="M10">
+        <v>0.25</v>
+      </c>
+      <c r="N10">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>1998</v>
+      </c>
+      <c r="C11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11">
+        <v>371</v>
+      </c>
+      <c r="G11">
+        <v>24</v>
+      </c>
+      <c r="H11" s="8">
+        <v>392</v>
+      </c>
+      <c r="I11">
+        <v>1.28</v>
+      </c>
+      <c r="J11">
+        <v>0.87</v>
+      </c>
+      <c r="K11">
+        <v>0.68</v>
+      </c>
+      <c r="L11">
+        <v>0.37</v>
+      </c>
+      <c r="M11">
+        <v>0.27</v>
+      </c>
+      <c r="N11">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12">
+        <v>2005</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12">
+        <v>306</v>
+      </c>
+      <c r="G12">
+        <v>24</v>
+      </c>
+      <c r="H12" s="8">
+        <v>433</v>
+      </c>
+      <c r="I12">
+        <v>0.74</v>
+      </c>
+      <c r="J12">
+        <v>0.63</v>
+      </c>
+      <c r="K12">
+        <v>0.85</v>
+      </c>
+      <c r="L12">
+        <v>0.26</v>
+      </c>
+      <c r="M12">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N12">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13">
+        <v>2006</v>
+      </c>
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13">
+        <v>942</v>
+      </c>
+      <c r="G13">
+        <v>24</v>
+      </c>
+      <c r="H13" s="8">
+        <v>1332</v>
+      </c>
+      <c r="I13">
+        <v>0.73</v>
+      </c>
+      <c r="J13">
+        <v>0.23</v>
+      </c>
+      <c r="K13">
+        <v>0.32</v>
+      </c>
+      <c r="L13">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="M13">
+        <v>0.17</v>
+      </c>
+      <c r="N13">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14">
+        <v>2009</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14">
+        <v>870</v>
+      </c>
+      <c r="G14">
+        <v>24</v>
+      </c>
+      <c r="H14" s="8">
+        <v>951</v>
+      </c>
+      <c r="I14">
+        <v>0.33</v>
+      </c>
+      <c r="J14">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="K14">
+        <v>0.42</v>
+      </c>
+      <c r="N14">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15">
+        <v>2009</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15">
+        <v>893</v>
+      </c>
+      <c r="G15">
+        <v>24</v>
+      </c>
+      <c r="H15" s="8">
+        <v>919</v>
+      </c>
+      <c r="I15">
+        <v>0.33</v>
+      </c>
+      <c r="J15">
+        <v>0.15</v>
+      </c>
+      <c r="K15">
+        <v>0.45</v>
+      </c>
+      <c r="N15">
+        <v>0.69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16">
+        <v>2009</v>
+      </c>
+      <c r="C16" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16">
+        <v>130</v>
+      </c>
+      <c r="G16">
+        <v>24</v>
+      </c>
+      <c r="H16" s="8">
+        <v>184</v>
+      </c>
+      <c r="I16">
+        <v>0.59</v>
+      </c>
+      <c r="J16">
+        <v>0.22</v>
+      </c>
+      <c r="K16">
+        <v>0.37</v>
+      </c>
+      <c r="L16">
+        <v>0.25</v>
+      </c>
+      <c r="M16">
+        <v>0.16</v>
+      </c>
+      <c r="N16">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17">
+        <v>2002</v>
+      </c>
+      <c r="C17" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17">
+        <v>802</v>
+      </c>
+      <c r="G17">
+        <v>36</v>
+      </c>
+      <c r="H17" s="8">
+        <v>1389</v>
+      </c>
+      <c r="I17">
+        <v>0.77</v>
+      </c>
+      <c r="J17">
+        <v>0.81</v>
+      </c>
+      <c r="K17">
+        <v>1.05</v>
+      </c>
+      <c r="L17">
+        <v>0.37</v>
+      </c>
+      <c r="M17">
+        <v>0.37</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18">
+        <v>2002</v>
+      </c>
+      <c r="C18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18">
+        <v>188</v>
+      </c>
+      <c r="G18">
+        <v>24</v>
+      </c>
+      <c r="H18" s="8">
+        <v>266</v>
+      </c>
+      <c r="I18">
+        <v>0.7</v>
+      </c>
+      <c r="J18">
+        <v>0.5</v>
+      </c>
+      <c r="K18">
+        <v>0.71</v>
+      </c>
+      <c r="L18">
+        <v>0.3</v>
+      </c>
+      <c r="M18">
+        <v>0.13</v>
+      </c>
+      <c r="N18">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19">
+        <v>2006</v>
+      </c>
+      <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" t="s">
+        <v>87</v>
+      </c>
+      <c r="F19">
+        <v>1171</v>
+      </c>
+      <c r="G19">
+        <v>24</v>
+      </c>
+      <c r="H19" s="8">
+        <v>1656</v>
+      </c>
+      <c r="I19">
+        <v>0.75</v>
+      </c>
+      <c r="J19">
+        <v>0.34</v>
+      </c>
+      <c r="K19">
+        <v>0.45</v>
+      </c>
+      <c r="L19">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="M19">
+        <v>0.23</v>
+      </c>
+      <c r="N19">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20">
+        <v>2008</v>
+      </c>
+      <c r="C20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20">
+        <v>223</v>
+      </c>
+      <c r="G20">
+        <v>36</v>
+      </c>
+      <c r="H20" s="8">
+        <v>292</v>
+      </c>
+      <c r="I20">
+        <v>0.36</v>
+      </c>
+      <c r="J20">
+        <v>0.11</v>
+      </c>
+      <c r="K20">
+        <v>0.31</v>
+      </c>
+      <c r="L20">
+        <v>0.26</v>
+      </c>
+      <c r="M20">
+        <v>0.09</v>
+      </c>
+      <c r="N20">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21">
+        <v>2008</v>
+      </c>
+      <c r="C21" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21">
+        <v>221</v>
+      </c>
+      <c r="G21">
+        <v>36</v>
+      </c>
+      <c r="H21" s="8">
+        <v>287</v>
+      </c>
+      <c r="I21">
+        <v>0.36</v>
+      </c>
+      <c r="J21">
+        <v>0.08</v>
+      </c>
+      <c r="K21">
+        <v>0.22</v>
+      </c>
+      <c r="L21">
+        <v>0.26</v>
+      </c>
+      <c r="M21">
+        <v>0.1</v>
+      </c>
+      <c r="N21">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22">
+        <v>2008</v>
+      </c>
+      <c r="C22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22">
+        <v>764</v>
+      </c>
+      <c r="G22">
+        <v>24</v>
+      </c>
+      <c r="H22" s="8">
+        <v>1080</v>
+      </c>
+      <c r="I22">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J22">
+        <v>0.3</v>
+      </c>
+      <c r="K22">
+        <v>1.03</v>
+      </c>
+      <c r="L22">
+        <v>0.09</v>
+      </c>
+      <c r="M22">
+        <v>0.12</v>
+      </c>
+      <c r="N22">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23">
+        <v>2009</v>
+      </c>
+      <c r="C23" t="s">
+        <v>103</v>
+      </c>
+      <c r="D23" t="s">
+        <v>109</v>
+      </c>
+      <c r="E23" t="s">
+        <v>91</v>
+      </c>
+      <c r="F23">
+        <v>118</v>
+      </c>
+      <c r="G23">
+        <v>24</v>
+      </c>
+      <c r="H23" s="8">
+        <v>129</v>
+      </c>
+      <c r="I23">
+        <v>1.05</v>
+      </c>
+      <c r="J23">
+        <v>0.91</v>
+      </c>
+      <c r="K23">
+        <v>0.87</v>
+      </c>
+      <c r="L23">
+        <v>0.17</v>
+      </c>
+      <c r="M23">
+        <v>0.21</v>
+      </c>
+      <c r="N23">
+        <v>1.24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24">
+        <v>2009</v>
+      </c>
+      <c r="C24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" t="s">
+        <v>92</v>
+      </c>
+      <c r="F24">
+        <v>123</v>
+      </c>
+      <c r="G24">
+        <v>24</v>
+      </c>
+      <c r="H24" s="8">
+        <v>123</v>
+      </c>
+      <c r="I24">
+        <v>1.05</v>
+      </c>
+      <c r="J24">
+        <v>0.73</v>
+      </c>
+      <c r="K24">
+        <v>0.7</v>
+      </c>
+      <c r="L24">
+        <v>0.17</v>
+      </c>
+      <c r="M24">
+        <v>0.18</v>
+      </c>
+      <c r="N24">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25">
+        <v>2009</v>
+      </c>
+      <c r="C25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" t="s">
+        <v>93</v>
+      </c>
+      <c r="F25">
+        <v>1345</v>
+      </c>
+      <c r="G25">
+        <v>24</v>
+      </c>
+      <c r="H25" s="8">
+        <v>1585</v>
+      </c>
+      <c r="I25">
+        <v>0.34</v>
+      </c>
+      <c r="J25">
+        <v>0.36</v>
+      </c>
+      <c r="K25">
+        <v>1.06</v>
+      </c>
+      <c r="L25">
+        <v>0.21</v>
+      </c>
+      <c r="M25">
+        <v>0.27</v>
+      </c>
+      <c r="N25">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26">
+        <v>2009</v>
+      </c>
+      <c r="C26" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26">
+        <v>1347</v>
+      </c>
+      <c r="G26">
+        <v>24</v>
+      </c>
+      <c r="H26" s="8">
+        <v>1588</v>
+      </c>
+      <c r="I26">
+        <v>0.34</v>
+      </c>
+      <c r="J26">
+        <v>0.33</v>
+      </c>
+      <c r="K26">
+        <v>0.97</v>
+      </c>
+      <c r="L26">
+        <v>0.21</v>
+      </c>
+      <c r="M26">
+        <v>0.22</v>
+      </c>
+      <c r="N26">
+        <v>1.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>